<commit_message>
Switch dashboard to 2026-27 Odd Semester labels and exports.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/details/All_Venue_Details.xlsx
+++ b/details/All_Venue_Details.xlsx
@@ -627,7 +627,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — All Programme Venue Summary (2025-26 Even Sem)</t>
+          <t>SRM Ramapuram — All Programme Venue Summary (2026-27 Odd Semester)</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6320,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Internet of Things — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Internet of Things — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -8989,7 +8989,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Electronics &amp; Communication Engg — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Electronics &amp; Communication Engg — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -11000,7 +11000,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Big Data Analytics &amp; Cloud Computing — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Big Data Analytics &amp; Cloud Computing — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -17683,7 +17683,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Information Technology — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Information Technology — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -22259,7 +22259,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — CSE (AI &amp; Machine Learning) — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — CSE (AI &amp; Machine Learning) — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -30660,7 +30660,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — CSE (Artificial Intelligence) — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — CSE (Artificial Intelligence) — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -32591,7 +32591,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Computer Science &amp; Engineering — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Computer Science &amp; Engineering — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -47160,7 +47160,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Cyber Security and Gaming Technology — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Cyber Security and Gaming Technology — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -55244,7 +55244,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Biotechnology — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Biotechnology — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -58110,7 +58110,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Biomedical Engineering — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Biomedical Engineering — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -61064,7 +61064,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Mechanical Engineering — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Mechanical Engineering — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -63838,7 +63838,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Civil Engineering — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Civil Engineering — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -66507,7 +66507,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Electrical &amp; Electronics Engineering — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Electrical &amp; Electronics Engineering — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>
@@ -68552,7 +68552,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SRM Ramapuram — Computer Science &amp; Business Systems — 2025-26 Even Sem</t>
+          <t>SRM Ramapuram — Computer Science &amp; Business Systems — 2026-27 Odd Semester</t>
         </is>
       </c>
     </row>

</xml_diff>